<commit_message>
Added simulation and mapping for distance to POIs --> Updated Template.
</commit_message>
<xml_diff>
--- a/Simulation Survey Data/results-survey581821.xlsx
+++ b/Simulation Survey Data/results-survey581821.xlsx
@@ -107,7 +107,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:IV2"/>
+  <dimension ref="A1:IZ2"/>
   <cols>
     <col collapsed="false" hidden="false" max="1024" min="1" style="0" customWidth="false" width="11.5"/>
   </cols>
@@ -780,615 +780,635 @@
       </c>
       <c r="ED1" s="0" t="inlineStr">
         <is>
+          <t>EntfernPOI[BStel]</t>
+        </is>
+      </c>
+      <c r="EE1" s="0" t="inlineStr">
+        <is>
+          <t>EntfernPOI[InBew]</t>
+        </is>
+      </c>
+      <c r="EF1" s="0" t="inlineStr">
+        <is>
+          <t>EntfernPOI[OutBew]</t>
+        </is>
+      </c>
+      <c r="EG1" s="0" t="inlineStr">
+        <is>
           <t>PhoneSystem</t>
         </is>
       </c>
-      <c r="EE1" s="0" t="inlineStr">
+      <c r="EH1" s="0" t="inlineStr">
         <is>
           <t>PhoneSystem[other]</t>
         </is>
       </c>
-      <c r="EF1" s="0" t="inlineStr">
+      <c r="EI1" s="0" t="inlineStr">
         <is>
           <t>AppUseGeneral</t>
         </is>
       </c>
-      <c r="EG1" s="0" t="inlineStr">
+      <c r="EJ1" s="0" t="inlineStr">
         <is>
           <t>QualAppGeneral</t>
         </is>
       </c>
-      <c r="EH1" s="0" t="inlineStr">
+      <c r="EK1" s="0" t="inlineStr">
         <is>
           <t>AppUseStudy</t>
         </is>
       </c>
-      <c r="EI1" s="0" t="inlineStr">
+      <c r="EL1" s="0" t="inlineStr">
         <is>
           <t>AppUseDays</t>
         </is>
       </c>
-      <c r="EJ1" s="0" t="inlineStr">
+      <c r="EM1" s="0" t="inlineStr">
         <is>
           <t>TransferAppDetail</t>
         </is>
       </c>
-      <c r="EK1" s="0" t="inlineStr">
+      <c r="EN1" s="0" t="inlineStr">
         <is>
           <t>TAM[WA1]</t>
         </is>
       </c>
-      <c r="EL1" s="0" t="inlineStr">
+      <c r="EO1" s="0" t="inlineStr">
         <is>
           <t>TAM[WA2]</t>
         </is>
       </c>
-      <c r="EM1" s="0" t="inlineStr">
+      <c r="EP1" s="0" t="inlineStr">
         <is>
           <t>TAM[WA3]</t>
         </is>
       </c>
-      <c r="EN1" s="0" t="inlineStr">
+      <c r="EQ1" s="0" t="inlineStr">
         <is>
           <t>TAM[WN1]</t>
         </is>
       </c>
-      <c r="EO1" s="0" t="inlineStr">
+      <c r="ER1" s="0" t="inlineStr">
         <is>
           <t>TAM[WN2]</t>
         </is>
       </c>
-      <c r="EP1" s="0" t="inlineStr">
+      <c r="ES1" s="0" t="inlineStr">
         <is>
           <t>TAM[WN3]</t>
         </is>
       </c>
-      <c r="EQ1" s="0" t="inlineStr">
+      <c r="ET1" s="0" t="inlineStr">
         <is>
           <t>TAM[WN4]</t>
         </is>
       </c>
-      <c r="ER1" s="0" t="inlineStr">
+      <c r="EU1" s="0" t="inlineStr">
         <is>
           <t>TAM[WB1]</t>
         </is>
       </c>
-      <c r="ES1" s="0" t="inlineStr">
+      <c r="EV1" s="0" t="inlineStr">
         <is>
           <t>TAM[WB2]</t>
         </is>
       </c>
-      <c r="ET1" s="0" t="inlineStr">
+      <c r="EW1" s="0" t="inlineStr">
         <is>
           <t>TAM[WB3]</t>
         </is>
       </c>
-      <c r="EU1" s="0" t="inlineStr">
+      <c r="EX1" s="0" t="inlineStr">
         <is>
           <t>TAM[WB4]</t>
         </is>
       </c>
-      <c r="EV1" s="0" t="inlineStr">
+      <c r="EY1" s="0" t="inlineStr">
         <is>
           <t>TAM[WF1]</t>
         </is>
       </c>
-      <c r="EW1" s="0" t="inlineStr">
+      <c r="EZ1" s="0" t="inlineStr">
         <is>
           <t>TAM[WF2]</t>
         </is>
       </c>
-      <c r="EX1" s="0" t="inlineStr">
+      <c r="FA1" s="0" t="inlineStr">
         <is>
           <t>TAM[WF3]</t>
         </is>
       </c>
-      <c r="EY1" s="0" t="inlineStr">
+      <c r="FB1" s="0" t="inlineStr">
         <is>
           <t>TAM[WF4]</t>
         </is>
       </c>
-      <c r="EZ1" s="0" t="inlineStr">
+      <c r="FC1" s="0" t="inlineStr">
         <is>
           <t>TAM[WV1]</t>
         </is>
       </c>
-      <c r="FA1" s="0" t="inlineStr">
+      <c r="FD1" s="0" t="inlineStr">
         <is>
           <t>TAM[WV2]</t>
         </is>
       </c>
-      <c r="FB1" s="0" t="inlineStr">
+      <c r="FE1" s="0" t="inlineStr">
         <is>
           <t>TAM[WV3]</t>
         </is>
       </c>
-      <c r="FC1" s="0" t="inlineStr">
+      <c r="FF1" s="0" t="inlineStr">
         <is>
           <t>TAM[WV4]</t>
         </is>
       </c>
-      <c r="FD1" s="0" t="inlineStr">
+      <c r="FG1" s="0" t="inlineStr">
         <is>
           <t>TAM[NI1]</t>
         </is>
       </c>
-      <c r="FE1" s="0" t="inlineStr">
+      <c r="FH1" s="0" t="inlineStr">
         <is>
           <t>TAM[NI2]</t>
         </is>
       </c>
-      <c r="FF1" s="0" t="inlineStr">
+      <c r="FI1" s="0" t="inlineStr">
         <is>
           <t>TAM[NI3]</t>
         </is>
       </c>
-      <c r="FG1" s="0" t="inlineStr">
+      <c r="FJ1" s="0" t="inlineStr">
         <is>
           <t>TAM[NI4]</t>
         </is>
       </c>
-      <c r="FH1" s="0" t="inlineStr">
+      <c r="FK1" s="0" t="inlineStr">
         <is>
           <t>QualPos</t>
         </is>
       </c>
-      <c r="FI1" s="0" t="inlineStr">
+      <c r="FL1" s="0" t="inlineStr">
         <is>
           <t>QualNeg</t>
         </is>
       </c>
-      <c r="FJ1" s="0" t="inlineStr">
+      <c r="FM1" s="0" t="inlineStr">
         <is>
           <t>otherAppUse</t>
         </is>
       </c>
-      <c r="FK1" s="0" t="inlineStr">
+      <c r="FN1" s="0" t="inlineStr">
         <is>
           <t>QualOthApp</t>
         </is>
       </c>
-      <c r="FL1" s="0" t="inlineStr">
+      <c r="FO1" s="0" t="inlineStr">
         <is>
           <t>SystemLink</t>
         </is>
       </c>
-      <c r="FM1" s="0" t="inlineStr">
+      <c r="FP1" s="0" t="inlineStr">
         <is>
           <t>eMailIG</t>
         </is>
       </c>
-      <c r="FN1" s="0" t="inlineStr">
+      <c r="FQ1" s="0" t="inlineStr">
         <is>
           <t>eMailValidIG</t>
         </is>
       </c>
-      <c r="FO1" s="0" t="inlineStr">
+      <c r="FR1" s="0" t="inlineStr">
         <is>
           <t>eMailKG</t>
         </is>
       </c>
-      <c r="FP1" s="0" t="inlineStr">
+      <c r="FS1" s="0" t="inlineStr">
         <is>
           <t>eMailValidKG</t>
         </is>
       </c>
-      <c r="FQ1" s="0" t="inlineStr">
+      <c r="FT1" s="0" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="FR1" s="0" t="inlineStr">
+      <c r="FU1" s="0" t="inlineStr">
         <is>
           <t>interviewtime</t>
         </is>
       </c>
-      <c r="FS1" s="0" t="inlineStr">
+      <c r="FV1" s="0" t="inlineStr">
         <is>
           <t>groupTime19488</t>
         </is>
       </c>
-      <c r="FT1" s="0" t="inlineStr">
+      <c r="FW1" s="0" t="inlineStr">
         <is>
           <t>timePointTime</t>
         </is>
       </c>
-      <c r="FU1" s="0" t="inlineStr">
+      <c r="FX1" s="0" t="inlineStr">
         <is>
           <t>groupTime19449</t>
         </is>
       </c>
-      <c r="FV1" s="0" t="inlineStr">
+      <c r="FY1" s="0" t="inlineStr">
         <is>
           <t>EinvTime</t>
         </is>
       </c>
-      <c r="FW1" s="0" t="inlineStr">
+      <c r="FZ1" s="0" t="inlineStr">
         <is>
           <t>groupTime19489</t>
         </is>
       </c>
-      <c r="FX1" s="0" t="inlineStr">
+      <c r="GA1" s="0" t="inlineStr">
         <is>
           <t>randomGroupTime</t>
         </is>
       </c>
-      <c r="FY1" s="0" t="inlineStr">
+      <c r="GB1" s="0" t="inlineStr">
         <is>
           <t>studyGroupTime</t>
         </is>
       </c>
-      <c r="FZ1" s="0" t="inlineStr">
+      <c r="GC1" s="0" t="inlineStr">
         <is>
           <t>AppNameTime</t>
         </is>
       </c>
-      <c r="GA1" s="0" t="inlineStr">
+      <c r="GD1" s="0" t="inlineStr">
         <is>
           <t>groupTime19452</t>
         </is>
       </c>
-      <c r="GB1" s="0" t="inlineStr">
+      <c r="GE1" s="0" t="inlineStr">
         <is>
           <t>Bew1Time</t>
         </is>
       </c>
-      <c r="GC1" s="0" t="inlineStr">
+      <c r="GF1" s="0" t="inlineStr">
         <is>
           <t>Bew2Time</t>
         </is>
       </c>
-      <c r="GD1" s="0" t="inlineStr">
+      <c r="GG1" s="0" t="inlineStr">
         <is>
           <t>Bew3Time</t>
         </is>
       </c>
-      <c r="GE1" s="0" t="inlineStr">
+      <c r="GH1" s="0" t="inlineStr">
         <is>
           <t>Bew4Time</t>
         </is>
       </c>
-      <c r="GF1" s="0" t="inlineStr">
+      <c r="GI1" s="0" t="inlineStr">
         <is>
           <t>Bew5Time</t>
         </is>
       </c>
-      <c r="GG1" s="0" t="inlineStr">
+      <c r="GJ1" s="0" t="inlineStr">
         <is>
           <t>Bew6Time</t>
         </is>
       </c>
-      <c r="GH1" s="0" t="inlineStr">
+      <c r="GK1" s="0" t="inlineStr">
         <is>
           <t>STGTime</t>
         </is>
       </c>
-      <c r="GI1" s="0" t="inlineStr">
+      <c r="GL1" s="0" t="inlineStr">
         <is>
           <t>groupTime19451</t>
         </is>
       </c>
-      <c r="GJ1" s="0" t="inlineStr">
+      <c r="GM1" s="0" t="inlineStr">
         <is>
           <t>HabitTime</t>
         </is>
       </c>
-      <c r="GK1" s="0" t="inlineStr">
+      <c r="GN1" s="0" t="inlineStr">
         <is>
           <t>groupTime19453</t>
         </is>
       </c>
-      <c r="GL1" s="0" t="inlineStr">
+      <c r="GO1" s="0" t="inlineStr">
         <is>
           <t>Intention1Time</t>
         </is>
       </c>
-      <c r="GM1" s="0" t="inlineStr">
+      <c r="GP1" s="0" t="inlineStr">
         <is>
           <t>Intention2Time</t>
         </is>
       </c>
-      <c r="GN1" s="0" t="inlineStr">
+      <c r="GQ1" s="0" t="inlineStr">
         <is>
           <t>Intention3Time</t>
         </is>
       </c>
-      <c r="GO1" s="0" t="inlineStr">
+      <c r="GR1" s="0" t="inlineStr">
         <is>
           <t>groupTime19454</t>
         </is>
       </c>
-      <c r="GP1" s="0" t="inlineStr">
+      <c r="GS1" s="0" t="inlineStr">
         <is>
           <t>Att1Time</t>
         </is>
       </c>
-      <c r="GQ1" s="0" t="inlineStr">
+      <c r="GT1" s="0" t="inlineStr">
         <is>
           <t>Att2Time</t>
         </is>
       </c>
-      <c r="GR1" s="0" t="inlineStr">
+      <c r="GU1" s="0" t="inlineStr">
         <is>
           <t>Att3Time</t>
         </is>
       </c>
-      <c r="GS1" s="0" t="inlineStr">
+      <c r="GV1" s="0" t="inlineStr">
         <is>
           <t>Att4Time</t>
         </is>
       </c>
-      <c r="GT1" s="0" t="inlineStr">
+      <c r="GW1" s="0" t="inlineStr">
         <is>
           <t>Att5Time</t>
         </is>
       </c>
-      <c r="GU1" s="0" t="inlineStr">
+      <c r="GX1" s="0" t="inlineStr">
         <is>
           <t>groupTime19455</t>
         </is>
       </c>
-      <c r="GV1" s="0" t="inlineStr">
+      <c r="GY1" s="0" t="inlineStr">
         <is>
           <t>Norm1Time</t>
         </is>
       </c>
-      <c r="GW1" s="0" t="inlineStr">
+      <c r="GZ1" s="0" t="inlineStr">
         <is>
           <t>Norm2Time</t>
         </is>
       </c>
-      <c r="GX1" s="0" t="inlineStr">
+      <c r="HA1" s="0" t="inlineStr">
         <is>
           <t>Norm3Time</t>
         </is>
       </c>
-      <c r="GY1" s="0" t="inlineStr">
+      <c r="HB1" s="0" t="inlineStr">
         <is>
           <t>ACheck1Time</t>
         </is>
       </c>
-      <c r="GZ1" s="0" t="inlineStr">
+      <c r="HC1" s="0" t="inlineStr">
         <is>
           <t>Norm4Time</t>
         </is>
       </c>
-      <c r="HA1" s="0" t="inlineStr">
+      <c r="HD1" s="0" t="inlineStr">
         <is>
           <t>Norm5Time</t>
         </is>
       </c>
-      <c r="HB1" s="0" t="inlineStr">
+      <c r="HE1" s="0" t="inlineStr">
         <is>
           <t>Norm6Time</t>
         </is>
       </c>
-      <c r="HC1" s="0" t="inlineStr">
+      <c r="HF1" s="0" t="inlineStr">
         <is>
           <t>groupTime19456</t>
         </is>
       </c>
-      <c r="HD1" s="0" t="inlineStr">
+      <c r="HG1" s="0" t="inlineStr">
         <is>
           <t>Control1Time</t>
         </is>
       </c>
-      <c r="HE1" s="0" t="inlineStr">
+      <c r="HH1" s="0" t="inlineStr">
         <is>
           <t>Control2Time</t>
         </is>
       </c>
-      <c r="HF1" s="0" t="inlineStr">
+      <c r="HI1" s="0" t="inlineStr">
         <is>
           <t>Control3Time</t>
         </is>
       </c>
-      <c r="HG1" s="0" t="inlineStr">
+      <c r="HJ1" s="0" t="inlineStr">
         <is>
           <t>Control4Time</t>
         </is>
       </c>
-      <c r="HH1" s="0" t="inlineStr">
+      <c r="HK1" s="0" t="inlineStr">
         <is>
           <t>groupTime19458</t>
         </is>
       </c>
-      <c r="HI1" s="0" t="inlineStr">
+      <c r="HL1" s="0" t="inlineStr">
         <is>
           <t>KIMTime</t>
         </is>
       </c>
-      <c r="HJ1" s="0" t="inlineStr">
+      <c r="HM1" s="0" t="inlineStr">
         <is>
           <t>groupTime19461</t>
         </is>
       </c>
-      <c r="HK1" s="0" t="inlineStr">
+      <c r="HN1" s="0" t="inlineStr">
         <is>
           <t>ZiMoTime</t>
         </is>
       </c>
-      <c r="HL1" s="0" t="inlineStr">
+      <c r="HO1" s="0" t="inlineStr">
         <is>
           <t>groupTime19862</t>
         </is>
       </c>
-      <c r="HM1" s="0" t="inlineStr">
+      <c r="HP1" s="0" t="inlineStr">
         <is>
           <t>MotivCompTime</t>
         </is>
       </c>
-      <c r="HN1" s="0" t="inlineStr">
+      <c r="HQ1" s="0" t="inlineStr">
         <is>
           <t>groupTime19863</t>
         </is>
       </c>
-      <c r="HO1" s="0" t="inlineStr">
+      <c r="HR1" s="0" t="inlineStr">
         <is>
           <t>VolSelfTime</t>
         </is>
       </c>
-      <c r="HP1" s="0" t="inlineStr">
+      <c r="HS1" s="0" t="inlineStr">
         <is>
           <t>groupTime19864</t>
         </is>
       </c>
-      <c r="HQ1" s="0" t="inlineStr">
+      <c r="HT1" s="0" t="inlineStr">
         <is>
           <t>ActionPlanTime</t>
         </is>
       </c>
-      <c r="HR1" s="0" t="inlineStr">
+      <c r="HU1" s="0" t="inlineStr">
         <is>
           <t>groupTime19450</t>
         </is>
       </c>
-      <c r="HS1" s="0" t="inlineStr">
+      <c r="HV1" s="0" t="inlineStr">
         <is>
           <t>GebTime</t>
         </is>
       </c>
-      <c r="HT1" s="0" t="inlineStr">
+      <c r="HW1" s="0" t="inlineStr">
         <is>
           <t>GesTime</t>
         </is>
       </c>
-      <c r="HU1" s="0" t="inlineStr">
+      <c r="HX1" s="0" t="inlineStr">
         <is>
           <t>EthnTime</t>
         </is>
       </c>
-      <c r="HV1" s="0" t="inlineStr">
+      <c r="HY1" s="0" t="inlineStr">
         <is>
           <t>WohnTime</t>
         </is>
       </c>
-      <c r="HW1" s="0" t="inlineStr">
+      <c r="HZ1" s="0" t="inlineStr">
         <is>
           <t>EduTime</t>
         </is>
       </c>
-      <c r="HX1" s="0" t="inlineStr">
+      <c r="IA1" s="0" t="inlineStr">
         <is>
           <t>ProfTime</t>
         </is>
       </c>
-      <c r="HY1" s="0" t="inlineStr">
+      <c r="IB1" s="0" t="inlineStr">
         <is>
           <t>EinkoTime</t>
         </is>
       </c>
-      <c r="HZ1" s="0" t="inlineStr">
+      <c r="IC1" s="0" t="inlineStr">
         <is>
           <t>BrancheTime</t>
         </is>
       </c>
-      <c r="IA1" s="0" t="inlineStr">
+      <c r="ID1" s="0" t="inlineStr">
         <is>
           <t>AlltagAblTime</t>
         </is>
       </c>
-      <c r="IB1" s="0" t="inlineStr">
+      <c r="IE1" s="0" t="inlineStr">
+        <is>
+          <t>EntfernPOITime</t>
+        </is>
+      </c>
+      <c r="IF1" s="0" t="inlineStr">
         <is>
           <t>PhoneSystemTime</t>
         </is>
       </c>
-      <c r="IC1" s="0" t="inlineStr">
+      <c r="IG1" s="0" t="inlineStr">
         <is>
           <t>AppUseGeneralTime</t>
         </is>
       </c>
-      <c r="ID1" s="0" t="inlineStr">
+      <c r="IH1" s="0" t="inlineStr">
         <is>
           <t>QualAppGeneralTime</t>
         </is>
       </c>
-      <c r="IE1" s="0" t="inlineStr">
+      <c r="II1" s="0" t="inlineStr">
         <is>
           <t>groupTime19487</t>
         </is>
       </c>
-      <c r="IF1" s="0" t="inlineStr">
+      <c r="IJ1" s="0" t="inlineStr">
         <is>
           <t>AppUseStudyTime</t>
         </is>
       </c>
-      <c r="IG1" s="0" t="inlineStr">
+      <c r="IK1" s="0" t="inlineStr">
         <is>
           <t>AppUseDaysTime</t>
         </is>
       </c>
-      <c r="IH1" s="0" t="inlineStr">
+      <c r="IL1" s="0" t="inlineStr">
         <is>
           <t>TransferAppDetailTime</t>
         </is>
       </c>
-      <c r="II1" s="0" t="inlineStr">
+      <c r="IM1" s="0" t="inlineStr">
         <is>
           <t>groupTime19486</t>
         </is>
       </c>
-      <c r="IJ1" s="0" t="inlineStr">
+      <c r="IN1" s="0" t="inlineStr">
         <is>
           <t>TAMTime</t>
         </is>
       </c>
-      <c r="IK1" s="0" t="inlineStr">
+      <c r="IO1" s="0" t="inlineStr">
         <is>
           <t>QualPosTime</t>
         </is>
       </c>
-      <c r="IL1" s="0" t="inlineStr">
+      <c r="IP1" s="0" t="inlineStr">
         <is>
           <t>QualNegTime</t>
         </is>
       </c>
-      <c r="IM1" s="0" t="inlineStr">
+      <c r="IQ1" s="0" t="inlineStr">
         <is>
           <t>groupTime19491</t>
         </is>
       </c>
-      <c r="IN1" s="0" t="inlineStr">
+      <c r="IR1" s="0" t="inlineStr">
         <is>
           <t>otherAppUseTime</t>
         </is>
       </c>
-      <c r="IO1" s="0" t="inlineStr">
+      <c r="IS1" s="0" t="inlineStr">
         <is>
           <t>QualOthAppTime</t>
         </is>
       </c>
-      <c r="IP1" s="0" t="inlineStr">
+      <c r="IT1" s="0" t="inlineStr">
         <is>
           <t>groupTime19462</t>
         </is>
       </c>
-      <c r="IQ1" s="0" t="inlineStr">
+      <c r="IU1" s="0" t="inlineStr">
         <is>
           <t>SystemLinkTime</t>
         </is>
       </c>
-      <c r="IR1" s="0" t="inlineStr">
+      <c r="IV1" s="0" t="inlineStr">
         <is>
           <t>eMailIGTime</t>
         </is>
       </c>
-      <c r="IS1" s="0" t="inlineStr">
+      <c r="IW1" s="0" t="inlineStr">
         <is>
           <t>eMailValidIGTime</t>
         </is>
       </c>
-      <c r="IT1" s="0" t="inlineStr">
+      <c r="IX1" s="0" t="inlineStr">
         <is>
           <t>eMailKGTime</t>
         </is>
       </c>
-      <c r="IU1" s="0" t="inlineStr">
+      <c r="IY1" s="0" t="inlineStr">
         <is>
           <t>eMailValidKGTime</t>
         </is>
       </c>
-      <c r="IV1" s="0" t="inlineStr">
+      <c r="IZ1" s="0" t="inlineStr">
         <is>
           <t>NameTime</t>
         </is>
@@ -1396,11 +1416,11 @@
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="2">
       <c r="A2" s="0" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026-03-24 09:55:00</t>
+          <t>2026-04-09 16:11:26</t>
         </is>
       </c>
       <c r="C2" s="0" t="n">
@@ -1412,16 +1432,16 @@
         </is>
       </c>
       <c r="E2" s="0" t="n">
-        <v>598916058</v>
+        <v>528927893</v>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>2026-03-24 09:52:21</t>
+          <t>2026-04-09 16:04:50</t>
         </is>
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-03-24 09:55:00</t>
+          <t>2026-04-09 16:11:26</t>
         </is>
       </c>
       <c r="H2" s="0"/>
@@ -1446,91 +1466,85 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t>3 Tage</t>
+          <t>1 Tag</t>
         </is>
       </c>
       <c r="O2" s="0" t="n">
-        <v>532</v>
+        <v>56</v>
       </c>
       <c r="P2" s="0" t="inlineStr">
         <is>
-          <t>3 Tage</t>
+          <t>4 Tage</t>
         </is>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>2 Tage</t>
+          <t>4 Tage</t>
         </is>
       </c>
       <c r="S2" s="0" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
           <t>Nein, aber ich plane in den nächsten 30 Tagen mit regelmässiger körperlicher Aktivität zu starten.</t>
         </is>
       </c>
-      <c r="U2" s="0" t="n">
+      <c r="U2" s="0" t="inlineStr">
+        <is>
+          <t>3 </t>
+        </is>
+      </c>
+      <c r="V2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="W2" s="0" t="inlineStr">
+        <is>
+          <t>3 </t>
+        </is>
+      </c>
+      <c r="X2" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="V2" s="0" t="inlineStr">
-        <is>
-          <t>2 </t>
-        </is>
-      </c>
-      <c r="W2" s="0" t="n">
+      <c r="Z2" s="0" t="inlineStr">
+        <is>
+          <t>3 </t>
+        </is>
+      </c>
+      <c r="AA2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB2" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="X2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="Y2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="Z2" s="0" t="n">
+      <c r="AC2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD2" s="0" t="n">
         <v>5</v>
-      </c>
-      <c r="AA2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="AB2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="AC2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="AD2" s="0" t="n">
-        <v>4</v>
       </c>
       <c r="AE2" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="AF2" s="0" t="n">
+      <c r="AF2" s="0" t="inlineStr">
+        <is>
+          <t>3 </t>
+        </is>
+      </c>
+      <c r="AG2" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="AG2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
       <c r="AH2" s="0" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AI2" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AJ2" s="0" t="inlineStr">
         <is>
@@ -1541,177 +1555,161 @@
         <v>5</v>
       </c>
       <c r="AL2" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM2" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="AM2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
       <c r="AN2" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO2" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP2" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ2" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="AO2" s="0" t="inlineStr">
-        <is>
-          <t>2 </t>
-        </is>
-      </c>
-      <c r="AP2" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="AQ2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
       <c r="AR2" s="0" t="inlineStr">
         <is>
+          <t>4 - stimmt völlig</t>
+        </is>
+      </c>
+      <c r="AS2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="AT2" s="0" t="inlineStr">
+        <is>
+          <t>0 - stimmt gar nicht</t>
+        </is>
+      </c>
+      <c r="AU2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="AV2" s="0" t="inlineStr">
+        <is>
+          <t>4 - stimmt völlig</t>
+        </is>
+      </c>
+      <c r="AW2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="AX2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="AY2" s="0" t="inlineStr">
+        <is>
           <t>3 - stimmt ziemlich</t>
         </is>
       </c>
-      <c r="AS2" s="0" t="inlineStr">
+      <c r="AZ2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="BA2" s="0" t="inlineStr">
+        <is>
+          <t>2 - stimmt teils-teils</t>
+        </is>
+      </c>
+      <c r="BB2" s="0" t="inlineStr">
         <is>
           <t>1 - stimmt wenig</t>
         </is>
       </c>
-      <c r="AT2" s="0" t="inlineStr">
-        <is>
-          <t>1 - stimmt wenig</t>
-        </is>
-      </c>
-      <c r="AU2" s="0" t="inlineStr">
-        <is>
-          <t>2 - stimmt teils-teils</t>
-        </is>
-      </c>
-      <c r="AV2" s="0" t="inlineStr">
-        <is>
-          <t>2 - stimmt teils-teils</t>
-        </is>
-      </c>
-      <c r="AW2" s="0" t="inlineStr">
-        <is>
-          <t>2 - stimmt teils-teils</t>
-        </is>
-      </c>
-      <c r="AX2" s="0" t="inlineStr">
-        <is>
-          <t>2 - stimmt teils-teils</t>
-        </is>
-      </c>
-      <c r="AY2" s="0" t="inlineStr">
+      <c r="BC2" s="0" t="inlineStr">
+        <is>
+          <t>4 - stimmt völlig</t>
+        </is>
+      </c>
+      <c r="BD2" s="0" t="inlineStr">
         <is>
           <t>3 - stimmt ziemlich</t>
         </is>
       </c>
-      <c r="AZ2" s="0" t="inlineStr">
-        <is>
-          <t>3 - stimmt ziemlich</t>
-        </is>
-      </c>
-      <c r="BA2" s="0" t="inlineStr">
-        <is>
-          <t>1 - stimmt wenig</t>
-        </is>
-      </c>
-      <c r="BB2" s="0" t="inlineStr">
-        <is>
-          <t>3 - stimmt ziemlich</t>
-        </is>
-      </c>
-      <c r="BC2" s="0" t="inlineStr">
-        <is>
-          <t>1 - stimmt wenig</t>
-        </is>
-      </c>
-      <c r="BD2" s="0" t="inlineStr">
-        <is>
-          <t>3 - stimmt ziemlich</t>
-        </is>
-      </c>
-      <c r="BE2" s="0" t="inlineStr">
+      <c r="BE2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF2" s="0" t="inlineStr">
         <is>
           <t>4 </t>
         </is>
       </c>
-      <c r="BF2" s="0" t="inlineStr">
+      <c r="BG2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH2" s="0" t="inlineStr">
         <is>
           <t>4 </t>
         </is>
       </c>
-      <c r="BG2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BI2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BJ2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BK2" s="0" t="inlineStr">
-        <is>
-          <t>1    ich stimme überhaupt nicht zu</t>
-        </is>
+      <c r="BI2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK2" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="BL2" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="BM2" s="0" t="inlineStr">
+      <c r="BM2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN2" s="0" t="inlineStr">
         <is>
           <t>4 </t>
-        </is>
-      </c>
-      <c r="BN2" s="0" t="inlineStr">
-        <is>
-          <t>1    ich stimme überhaupt nicht zu</t>
         </is>
       </c>
       <c r="BO2" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="BP2" s="0" t="n">
+      <c r="BP2" s="0" t="inlineStr">
+        <is>
+          <t>4 </t>
+        </is>
+      </c>
+      <c r="BQ2" s="0" t="inlineStr">
+        <is>
+          <t>5    ich stimme voll und ganz zu</t>
+        </is>
+      </c>
+      <c r="BR2" s="0" t="inlineStr">
+        <is>
+          <t>1    ich stimme überhaupt nicht zu</t>
+        </is>
+      </c>
+      <c r="BS2" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="BQ2" s="0" t="n">
+      <c r="BT2" s="0" t="inlineStr">
+        <is>
+          <t>4 </t>
+        </is>
+      </c>
+      <c r="BU2" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="BR2" s="0" t="inlineStr">
-        <is>
-          <t>1    ich stimme überhaupt nicht zu</t>
-        </is>
-      </c>
-      <c r="BS2" s="0" t="inlineStr">
+      <c r="BV2" s="0" t="inlineStr">
+        <is>
+          <t>5    ich stimme voll und ganz zu</t>
+        </is>
+      </c>
+      <c r="BW2" s="0" t="inlineStr">
         <is>
           <t>4 </t>
-        </is>
-      </c>
-      <c r="BT2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BU2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BV2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
-      </c>
-      <c r="BW2" s="0" t="inlineStr">
-        <is>
-          <t>5    ich stimme voll und ganz zu</t>
         </is>
       </c>
       <c r="BX2" s="0" t="n">
@@ -1729,33 +1727,31 @@
         <v>3</v>
       </c>
       <c r="CB2" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CC2" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="CD2" s="0" t="inlineStr">
-        <is>
-          <t>4 </t>
-        </is>
+      <c r="CD2" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="CE2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="CF2" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="CF2" s="0" t="n">
+      <c r="CG2" s="0" t="inlineStr">
+        <is>
+          <t>5    ich stimme voll und ganz zu</t>
+        </is>
+      </c>
+      <c r="CH2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI2" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="CG2" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="CH2" s="0" t="inlineStr">
-        <is>
-          <t>1    ich stimme überhaupt nicht zu</t>
-        </is>
-      </c>
-      <c r="CI2" s="0" t="n">
-        <v>3</v>
-      </c>
       <c r="CJ2" s="0" t="inlineStr">
         <is>
           <t>3 </t>
@@ -1763,51 +1759,49 @@
       </c>
       <c r="CK2" s="0" t="inlineStr">
         <is>
+          <t>1     trifft nicht zu</t>
+        </is>
+      </c>
+      <c r="CL2" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="CM2" s="0" t="inlineStr">
+        <is>
+          <t>3 </t>
+        </is>
+      </c>
+      <c r="CN2" s="0" t="inlineStr">
+        <is>
           <t>2 </t>
         </is>
       </c>
-      <c r="CL2" s="0" t="inlineStr">
+      <c r="CO2" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="CP2" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="CQ2" s="0" t="inlineStr">
         <is>
           <t>3 </t>
         </is>
       </c>
-      <c r="CM2" s="0" t="inlineStr">
+      <c r="CR2" s="0" t="inlineStr">
         <is>
           <t>3 </t>
         </is>
       </c>
-      <c r="CN2" s="0" t="n">
+      <c r="CS2" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="CO2" s="0" t="inlineStr">
+      <c r="CT2" s="0" t="inlineStr">
         <is>
           <t>2 </t>
         </is>
       </c>
-      <c r="CP2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="CQ2" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="CR2" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="CS2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
-      <c r="CT2" s="0" t="inlineStr">
-        <is>
-          <t>3 </t>
-        </is>
-      </c>
       <c r="CU2" s="0" t="inlineStr">
         <is>
-          <t>2008-03-05 00:00:00</t>
+          <t>2000-03-31 00:00:00</t>
         </is>
       </c>
       <c r="CV2" s="0" t="inlineStr">
@@ -1830,13 +1824,13 @@
       <c r="DA2" s="0"/>
       <c r="DB2" s="0" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nein</t>
         </is>
       </c>
       <c r="DC2" s="0"/>
       <c r="DD2" s="0" t="inlineStr">
         <is>
-          <t>Nein</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="DE2" s="0"/>
@@ -1879,75 +1873,81 @@
       </c>
       <c r="DS2" s="0" t="inlineStr">
         <is>
-          <t>Selbständig</t>
+          <t>Studium</t>
         </is>
       </c>
       <c r="DT2" s="0"/>
       <c r="DU2" s="0" t="inlineStr">
         <is>
-          <t>4500-5000 CHF</t>
+          <t>1000 - 1500 CHF</t>
         </is>
       </c>
       <c r="DV2" s="0"/>
       <c r="DW2" s="0" t="inlineStr">
         <is>
-          <t>Bürojob sitzend</t>
+          <t>Bürojob oft sitzend</t>
         </is>
       </c>
       <c r="DX2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="DY2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="DZ2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="EA2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="EB2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="EC2" s="0" t="inlineStr">
         <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="ED2" s="0" t="inlineStr">
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="ED2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="EE2" s="0" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="EF2" s="0" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="EG2" s="0" t="inlineStr">
         <is>
           <t>Android</t>
         </is>
       </c>
-      <c r="EE2" s="0"/>
-      <c r="EF2" s="0" t="inlineStr">
+      <c r="EH2" s="0"/>
+      <c r="EI2" s="0" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="EG2" s="0" t="inlineStr">
-        <is>
-          <t>Samsung Watch</t>
-        </is>
-      </c>
-      <c r="EH2" s="0" t="inlineStr">
+      <c r="EJ2" s="0" t="inlineStr">
+        <is>
+          <t>Oura Ring</t>
+        </is>
+      </c>
+      <c r="EK2" s="0" t="inlineStr">
         <is>
           <t>N. v.</t>
         </is>
       </c>
-      <c r="EI2" s="0"/>
-      <c r="EJ2" s="0"/>
-      <c r="EK2" s="0"/>
       <c r="EL2" s="0"/>
       <c r="EM2" s="0"/>
       <c r="EN2" s="0"/>
@@ -1972,118 +1972,118 @@
       <c r="FG2" s="0"/>
       <c r="FH2" s="0"/>
       <c r="FI2" s="0"/>
-      <c r="FJ2" s="0" t="inlineStr">
+      <c r="FJ2" s="0"/>
+      <c r="FK2" s="0"/>
+      <c r="FL2" s="0"/>
+      <c r="FM2" s="0" t="inlineStr">
         <is>
           <t>N. v.</t>
         </is>
       </c>
-      <c r="FK2" s="0"/>
-      <c r="FL2" s="0" t="inlineStr">
+      <c r="FN2" s="0"/>
+      <c r="FO2" s="0" t="inlineStr">
         <is>
           <t>if(timePoint == 1,   if(PhoneSystem == "Googl", "Android: https://play.google.com/store/apps/details?id=ai.gymian.alife",    if(PhoneSystem == "Apple", "iOS: https://apps.apple.com/ch/app/alife-dein-ki-coach/id6756587565", "Android: https://play.google.com/store/apps/details?id=ai.gymian.alife | iOS: https://apps.apple.com/ch/app/alife-dein-ki-coach/id6756587565"   )  ),   if(TOKEN:ATTRIBUTE_2 == "Googl", "Android: https://play.google.com/store/apps/details?id=ai.gymian.alife",    if(TOKEN:ATTRIBUTE_2 == "Apple", "iOS: https://apps.apple.com/ch/app/alife-dein-ki-coach/id6756587565", "Android: https://play.google.com/store/apps/details?id=ai.gymian.alife | iOS: https://apps.apple.com/ch/app/alife-dein-ki-coach/id6756587565"   )  ) )</t>
         </is>
       </c>
-      <c r="FM2" s="0" t="inlineStr">
-        <is>
-          <t>test@test.ch</t>
-        </is>
-      </c>
-      <c r="FN2" s="0" t="inlineStr">
-        <is>
-          <t>test@test.ch</t>
-        </is>
-      </c>
-      <c r="FO2" s="0"/>
-      <c r="FP2" s="0"/>
+      <c r="FP2" s="0" t="inlineStr">
+        <is>
+          <t>peter.meier@gmx.ch</t>
+        </is>
+      </c>
       <c r="FQ2" s="0" t="inlineStr">
         <is>
-          <t>Peter</t>
-        </is>
-      </c>
-      <c r="FR2" s="0" t="n">
-        <v>166.85</v>
-      </c>
+          <t>peter.meier@gmx.ch</t>
+        </is>
+      </c>
+      <c r="FR2" s="0"/>
       <c r="FS2" s="0"/>
-      <c r="FT2" s="0"/>
+      <c r="FT2" s="0" t="inlineStr">
+        <is>
+          <t>peter4573x</t>
+        </is>
+      </c>
       <c r="FU2" s="0" t="n">
-        <v>3.3</v>
+        <v>404.16</v>
       </c>
       <c r="FV2" s="0"/>
       <c r="FW2" s="0"/>
-      <c r="FX2" s="0"/>
+      <c r="FX2" s="0" t="n">
+        <v>6.1</v>
+      </c>
       <c r="FY2" s="0"/>
       <c r="FZ2" s="0"/>
-      <c r="GA2" s="0" t="n">
-        <v>11.48</v>
-      </c>
+      <c r="GA2" s="0"/>
       <c r="GB2" s="0"/>
       <c r="GC2" s="0"/>
-      <c r="GD2" s="0"/>
+      <c r="GD2" s="0" t="n">
+        <v>25.9</v>
+      </c>
       <c r="GE2" s="0"/>
       <c r="GF2" s="0"/>
       <c r="GG2" s="0"/>
       <c r="GH2" s="0"/>
-      <c r="GI2" s="0" t="n">
-        <v>5.39</v>
-      </c>
+      <c r="GI2" s="0"/>
       <c r="GJ2" s="0"/>
-      <c r="GK2" s="0" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="GL2" s="0"/>
+      <c r="GK2" s="0"/>
+      <c r="GL2" s="0" t="n">
+        <v>7.63</v>
+      </c>
       <c r="GM2" s="0"/>
-      <c r="GN2" s="0"/>
-      <c r="GO2" s="0" t="n">
-        <v>7.39</v>
-      </c>
+      <c r="GN2" s="0" t="n">
+        <v>15.72</v>
+      </c>
+      <c r="GO2" s="0"/>
       <c r="GP2" s="0"/>
       <c r="GQ2" s="0"/>
-      <c r="GR2" s="0"/>
+      <c r="GR2" s="0" t="n">
+        <v>8.61</v>
+      </c>
       <c r="GS2" s="0"/>
       <c r="GT2" s="0"/>
-      <c r="GU2" s="0" t="n">
-        <v>9.67</v>
-      </c>
+      <c r="GU2" s="0"/>
       <c r="GV2" s="0"/>
       <c r="GW2" s="0"/>
-      <c r="GX2" s="0"/>
+      <c r="GX2" s="0" t="n">
+        <v>19.9</v>
+      </c>
       <c r="GY2" s="0"/>
       <c r="GZ2" s="0"/>
       <c r="HA2" s="0"/>
       <c r="HB2" s="0"/>
-      <c r="HC2" s="0" t="n">
-        <v>6.28</v>
-      </c>
+      <c r="HC2" s="0"/>
       <c r="HD2" s="0"/>
       <c r="HE2" s="0"/>
-      <c r="HF2" s="0"/>
+      <c r="HF2" s="0" t="n">
+        <v>10.47</v>
+      </c>
       <c r="HG2" s="0"/>
-      <c r="HH2" s="0" t="n">
-        <v>22.35</v>
-      </c>
+      <c r="HH2" s="0"/>
       <c r="HI2" s="0"/>
-      <c r="HJ2" s="0" t="n">
-        <v>31.47</v>
-      </c>
-      <c r="HK2" s="0"/>
-      <c r="HL2" s="0" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="HM2" s="0"/>
-      <c r="HN2" s="0" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="HO2" s="0"/>
-      <c r="HP2" s="0" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="HQ2" s="0"/>
-      <c r="HR2" s="0" t="n">
-        <v>34.44</v>
-      </c>
-      <c r="HS2" s="0"/>
+      <c r="HJ2" s="0"/>
+      <c r="HK2" s="0" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="HL2" s="0"/>
+      <c r="HM2" s="0" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="HN2" s="0"/>
+      <c r="HO2" s="0" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="HP2" s="0"/>
+      <c r="HQ2" s="0" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="HR2" s="0"/>
+      <c r="HS2" s="0" t="n">
+        <v>23.83</v>
+      </c>
       <c r="HT2" s="0"/>
-      <c r="HU2" s="0"/>
+      <c r="HU2" s="0" t="n">
+        <v>134.67</v>
+      </c>
       <c r="HV2" s="0"/>
       <c r="HW2" s="0"/>
       <c r="HX2" s="0"/>
@@ -2104,15 +2104,19 @@
       <c r="IM2" s="0"/>
       <c r="IN2" s="0"/>
       <c r="IO2" s="0"/>
-      <c r="IP2" s="0" t="n">
-        <v>16.87</v>
-      </c>
+      <c r="IP2" s="0"/>
       <c r="IQ2" s="0"/>
       <c r="IR2" s="0"/>
       <c r="IS2" s="0"/>
-      <c r="IT2" s="0"/>
+      <c r="IT2" s="0" t="n">
+        <v>81.52</v>
+      </c>
       <c r="IU2" s="0"/>
       <c r="IV2" s="0"/>
+      <c r="IW2" s="0"/>
+      <c r="IX2" s="0"/>
+      <c r="IY2" s="0"/>
+      <c r="IZ2" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>